<commit_message>
test(envmon): nysdec R6 fixture creates real same-sample date ambiguity
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LKGk2CE9hoaSVDn56WMBaC
</commit_message>
<xml_diff>
--- a/tests/fixtures/nysdec_edd_fixture.xlsx
+++ b/tests/fixtures/nysdec_edd_fixture.xlsx
@@ -985,7 +985,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>N-002</t>
+          <t>N-001</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1045,22 +1045,22 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>LAB-N-002</t>
+          <t>LAB-N-001</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>7439-92-1</t>
+          <t>7440-50-8</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Lead</t>
+          <t>Copper</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>8.1</t>
+          <t>3.2</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -1395,7 +1395,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>N-002</t>
+          <t>N-001</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">

</xml_diff>